<commit_message>
04: tighten readme/starter wording around gpai provider framing, tier coverage, and regulation provenance; complete the starter matrix row-14 templates.
</commit_message>
<xml_diff>
--- a/04_regulatory-compliance-for-ai-eu-ai-act/exercises/starter/compliance_plan.xlsx
+++ b/04_regulatory-compliance-for-ai-eu-ai-act/exercises/starter/compliance_plan.xlsx
@@ -155,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -200,6 +200,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1481,22 +1487,22 @@
       </c>
     </row>
     <row r="14" ht="100" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>REQ-013</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Serious-Incident Reporting — Notify national competent authority of serious incidents per Article 73 (enforces Aug 2026)</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Article 73</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>High-Risk</t>
         </is>
@@ -1519,6 +1525,21 @@
       <c r="H14" s="16" t="inlineStr">
         <is>
           <t>[Your response here — describe the gap and plan the 15-day reporting SLA plus designated notifying-authority lead; consider integration with the M6 incident-response work.]</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="inlineStr">
+        <is>
+          <t>[Your response here — outline the remediation plan (15-day reporting SLA, escalation path, integration with incident detection).]</t>
+        </is>
+      </c>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>[Your response here — name the accountable function (e.g., DPO, Compliance, Incident Response).]</t>
+        </is>
+      </c>
+      <c r="K14" s="19" t="inlineStr">
+        <is>
+          <t>[Your response here — pick a realistic target date before Aug 2026 (YYYY-MM-DD).]</t>
         </is>
       </c>
     </row>
@@ -2283,17 +2304,17 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>General-Purpose AI models — including those with systemic risk. Added in 2026 EU AI Act refresh.</t>
+          <t>General-Purpose AI models — including those with systemic risk. Introduced by Regulation (EU) 2024/1689; obligations applicable from 2 Aug 2025.</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>Foundation-model APIs embedded in customer-facing assistants, chatbots, code copilots, RAG systems.</t>
+          <t>Providers of general-purpose foundation models — e.g. models offered via API that power customer-facing assistants, chatbots, code copilots, RAG systems.</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>Transparency to downstream deployers (Art. 53), copyright disclosure, technical documentation; if systemic risk, additional model evaluation + adversarial testing + Art. 55 obligations.</t>
+          <t>Provider obligations — transparency to downstream deployers (Art. 53), copyright disclosure, technical documentation; if systemic risk, additional model evaluation + adversarial testing + Art. 55 obligations.</t>
         </is>
       </c>
     </row>

</xml_diff>